<commit_message>
Removed lock from Kicad Files
</commit_message>
<xml_diff>
--- a/Purchasing/BOM/Ultimate BOM.xlsx
+++ b/Purchasing/BOM/Ultimate BOM.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elijahrobinson/Documents/GitHub/Robot-Dog/Purchasing/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFD764F3-005F-6F40-A280-338C34DD7981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC9A2B99-3C50-4547-AB8C-86AC7DE28C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="920" windowWidth="29240" windowHeight="16880" xr2:uid="{B7364A64-1EA0-9049-A7FC-B4FA1E16182F}"/>
   </bookViews>
   <sheets>
     <sheet name="Total Price" sheetId="4" r:id="rId1"/>
-    <sheet name="Cycloidal Gearbox" sheetId="1" r:id="rId2"/>
-    <sheet name="FOC PCB" sheetId="2" r:id="rId3"/>
-    <sheet name="Leg Assembly" sheetId="3" r:id="rId4"/>
+    <sheet name="Body Assembly" sheetId="6" r:id="rId2"/>
+    <sheet name="Cycloidal Gearbox" sheetId="1" r:id="rId3"/>
+    <sheet name="FOC PCB" sheetId="2" r:id="rId4"/>
+    <sheet name="Leg Assembly" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="220">
   <si>
     <t>ITEM NO.</t>
   </si>
@@ -675,6 +676,30 @@
   </si>
   <si>
     <t>3D Printer Filament</t>
+  </si>
+  <si>
+    <t>Carbon Fiber Rods</t>
+  </si>
+  <si>
+    <t>https://a.co/d/098f3vCr</t>
+  </si>
+  <si>
+    <t>600MM Length Carbon Fiber Tube</t>
+  </si>
+  <si>
+    <t>Body Assembly</t>
+  </si>
+  <si>
+    <t>Funding Money</t>
+  </si>
+  <si>
+    <t>Who</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Chad Robinson</t>
   </si>
 </sst>
 </file>
@@ -840,7 +865,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -908,6 +933,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -941,17 +974,11 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -962,30 +989,38 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill>
@@ -1351,7 +1386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C4E62B7-8324-4D43-A746-C69356B7E16F}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.33203125" customWidth="1"/>
@@ -1398,7 +1433,7 @@
         <f>'Cycloidal Gearbox'!I28</f>
         <v>81.931542499999978</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="28">
         <v>12</v>
       </c>
       <c r="E2" s="25">
@@ -1431,11 +1466,11 @@
         <f>'Leg Assembly'!I25</f>
         <v>42.425021999999984</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="28">
         <v>12</v>
       </c>
       <c r="E3" s="25">
-        <f t="shared" ref="E3:E6" si="0">C3*D3</f>
+        <f t="shared" ref="E3:E7" si="0">C3*D3</f>
         <v>509.10026399999981</v>
       </c>
       <c r="G3" s="1">
@@ -1464,7 +1499,7 @@
         <f>'FOC PCB'!I41</f>
         <v>38.513933333333327</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="28">
         <v>12</v>
       </c>
       <c r="E4" s="25">
@@ -1496,7 +1531,7 @@
       <c r="C5" s="5">
         <v>8</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="28">
         <v>1</v>
       </c>
       <c r="E5" s="25">
@@ -1527,12 +1562,12 @@
       <c r="C6" s="5">
         <v>15</v>
       </c>
-      <c r="D6" s="1">
-        <v>3</v>
+      <c r="D6" s="28">
+        <v>4</v>
       </c>
       <c r="E6" s="25">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="G6" s="1">
         <v>5</v>
@@ -1542,33 +1577,91 @@
       <c r="J6" s="5"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C7" s="5">
+        <f>'Body Assembly'!L12</f>
+        <v>500</v>
+      </c>
+      <c r="D7" s="28">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25">
+        <f t="shared" si="0"/>
+        <v>500</v>
+      </c>
+      <c r="G7" s="1">
+        <v>6</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="29"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="13">
-        <f>SUM(E2:E6)</f>
-        <v>2007.4459739999993</v>
-      </c>
-      <c r="G7" s="30" t="s">
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="13">
+        <f>SUM(E2:E7)</f>
+        <v>2522.4459739999993</v>
+      </c>
+      <c r="G8" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="H7" s="31"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="13">
+      <c r="H8" s="35"/>
+      <c r="I8" s="36"/>
+      <c r="J8" s="13">
         <f>SUM(J2:J6)</f>
         <v>865.70788799999991</v>
       </c>
     </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="B16" s="57"/>
+      <c r="C16" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="57" t="s">
+        <v>219</v>
+      </c>
+      <c r="B17" s="57"/>
+      <c r="C17" s="5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="G7:I7"/>
+  <mergeCells count="5">
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A15:C15"/>
   </mergeCells>
-  <conditionalFormatting sqref="A2:E6 G2:J6">
-    <cfRule type="expression" dxfId="5" priority="2">
+  <conditionalFormatting sqref="G2:J7 A2:E7">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>MOD(ROW(),2)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1577,6 +1670,292 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{257BEE17-54E8-714C-9FC2-0AAD6BDD2F44}">
+  <dimension ref="A1:L46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="33.33203125" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" customWidth="1"/>
+    <col min="4" max="4" width="57.5" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="17.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="15" max="18" width="10.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="53" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="14">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="55"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="25"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="25"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="25"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="25"/>
+    </row>
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="D7" s="53" t="s">
+        <v>213</v>
+      </c>
+      <c r="E7" s="9">
+        <v>25</v>
+      </c>
+      <c r="F7" s="6">
+        <v>2</v>
+      </c>
+      <c r="G7" s="8">
+        <f>E7/F7</f>
+        <v>12.5</v>
+      </c>
+      <c r="H7" s="6">
+        <v>2</v>
+      </c>
+      <c r="I7" s="8">
+        <f>G7*H7</f>
+        <v>25</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1">
+        <v>4</v>
+      </c>
+      <c r="L7" s="25">
+        <f>K7*G7</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="25"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="25"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="25"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="25">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="13">
+        <f>SUM(I2:I10)</f>
+        <v>25</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="K12" s="37"/>
+      <c r="L12" s="23">
+        <f>SUM(L2:L11)</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="I16" s="30"/>
+    </row>
+    <row r="43" ht="31" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" ht="32" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" ht="32" customHeight="1" x14ac:dyDescent="0.2"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="J12:K12"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A2:L11">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>MOD(ROW(),2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="D7" r:id="rId1" xr:uid="{57B4361D-48E2-3B41-B418-FE89579F184B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BCE8930-9406-2043-8E02-400D939E2382}">
   <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1635,13 +2014,13 @@
       <c r="B2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="34">
+      <c r="E2" s="38">
         <v>29.98</v>
       </c>
       <c r="F2" s="11">
@@ -1663,7 +2042,7 @@
         <v>12</v>
       </c>
       <c r="L2" s="25">
-        <f>(IF(K2-J2&lt;0,0,K2-J2))*G2</f>
+        <f t="shared" ref="L2:L27" si="0">(IF(K2-J2&lt;0,0,K2-J2))*G2</f>
         <v>4.9610000000000003</v>
       </c>
     </row>
@@ -1674,9 +2053,9 @@
       <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="34"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="38"/>
       <c r="F3" s="6">
         <v>3.0099999999999998E-2</v>
       </c>
@@ -1696,7 +2075,7 @@
         <v>12</v>
       </c>
       <c r="L3" s="25">
-        <f>(IF(K3-J3&lt;0,0,K3-J3))*G3</f>
+        <f t="shared" si="0"/>
         <v>4.9610000000000003</v>
       </c>
     </row>
@@ -1707,9 +2086,9 @@
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="34"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="38"/>
       <c r="F4" s="6">
         <v>1.15E-2</v>
       </c>
@@ -1729,7 +2108,7 @@
         <v>24</v>
       </c>
       <c r="L4" s="25">
-        <f>(IF(K4-J4&lt;0,0,K4-J4))*G4</f>
+        <f t="shared" si="0"/>
         <v>3.7839999999999998</v>
       </c>
     </row>
@@ -1740,9 +2119,9 @@
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="34"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="38"/>
       <c r="F5" s="6">
         <v>3.5999999999999999E-3</v>
       </c>
@@ -1762,7 +2141,7 @@
         <v>12</v>
       </c>
       <c r="L5" s="25">
-        <f>(IF(K5-J5&lt;0,0,K5-J5))*G5</f>
+        <f t="shared" si="0"/>
         <v>0.59399999999999997</v>
       </c>
     </row>
@@ -1773,9 +2152,9 @@
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="34"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="38"/>
       <c r="F6" s="6">
         <v>2.0000000000000001E-4</v>
       </c>
@@ -1795,7 +2174,7 @@
         <v>12</v>
       </c>
       <c r="L6" s="25">
-        <f>(IF(K6-J6&lt;0,0,K6-J6))*G6</f>
+        <f t="shared" si="0"/>
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
@@ -1806,9 +2185,9 @@
       <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="34"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="38"/>
       <c r="F7" s="6">
         <v>4.0000000000000002E-4</v>
       </c>
@@ -1828,7 +2207,7 @@
         <v>12</v>
       </c>
       <c r="L7" s="25">
-        <f>(IF(K7-J7&lt;0,0,K7-J7))*G7</f>
+        <f t="shared" si="0"/>
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
@@ -1839,9 +2218,9 @@
       <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="34"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="38"/>
       <c r="F8" s="6">
         <v>4.2200000000000001E-2</v>
       </c>
@@ -1861,7 +2240,7 @@
         <v>12</v>
       </c>
       <c r="L8" s="25">
-        <f>(IF(K8-J8&lt;0,0,K8-J8))*G8</f>
+        <f t="shared" si="0"/>
         <v>6.9630000000000001</v>
       </c>
     </row>
@@ -1872,9 +2251,9 @@
       <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="34"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="38"/>
       <c r="F9" s="6">
         <v>5.0000000000000001E-4</v>
       </c>
@@ -1894,7 +2273,7 @@
         <v>12</v>
       </c>
       <c r="L9" s="25">
-        <f>(IF(K9-J9&lt;0,0,K9-J9))*G9</f>
+        <f t="shared" si="0"/>
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
@@ -1905,9 +2284,9 @@
       <c r="B10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="34"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="38"/>
       <c r="F10" s="6">
         <v>3.2000000000000002E-3</v>
       </c>
@@ -1927,7 +2306,7 @@
         <v>12</v>
       </c>
       <c r="L10" s="25">
-        <f>(IF(K10-J10&lt;0,0,K10-J10))*G10</f>
+        <f t="shared" si="0"/>
         <v>0.53900000000000003</v>
       </c>
     </row>
@@ -1938,9 +2317,9 @@
       <c r="B11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="34"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="38"/>
       <c r="F11" s="6">
         <v>1E-4</v>
       </c>
@@ -1960,7 +2339,7 @@
         <v>48</v>
       </c>
       <c r="L11" s="25">
-        <f>(IF(K11-J11&lt;0,0,K11-J11))*G11</f>
+        <f t="shared" si="0"/>
         <v>8.7999999999999995E-2</v>
       </c>
     </row>
@@ -1971,9 +2350,9 @@
       <c r="B12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="38"/>
       <c r="F12" s="6">
         <v>1.2500000000000001E-2</v>
       </c>
@@ -1993,7 +2372,7 @@
         <v>12</v>
       </c>
       <c r="L12" s="25">
-        <f>(IF(K12-J12&lt;0,0,K12-J12))*G12</f>
+        <f t="shared" si="0"/>
         <v>2.0680000000000001</v>
       </c>
     </row>
@@ -2004,9 +2383,9 @@
       <c r="B13" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="35"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="39"/>
       <c r="F13" s="6">
         <v>1.95E-2</v>
       </c>
@@ -2026,7 +2405,7 @@
         <v>12</v>
       </c>
       <c r="L13" s="25">
-        <f>(IF(K13-J13&lt;0,0,K13-J13))*G13</f>
+        <f t="shared" si="0"/>
         <v>3.2229999999999999</v>
       </c>
     </row>
@@ -2065,7 +2444,7 @@
         <v>24</v>
       </c>
       <c r="L14" s="25">
-        <f>(IF(K14-J14&lt;0,0,K14-J14))*G14</f>
+        <f t="shared" si="0"/>
         <v>53.371000000000002</v>
       </c>
     </row>
@@ -2104,7 +2483,7 @@
         <v>72</v>
       </c>
       <c r="L15" s="25">
-        <f>(IF(K15-J15&lt;0,0,K15-J15))*G15</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2143,7 +2522,7 @@
         <v>24</v>
       </c>
       <c r="L16" s="25">
-        <f>(IF(K16-J16&lt;0,0,K16-J16))*G16</f>
+        <f t="shared" si="0"/>
         <v>8.5579999999999998</v>
       </c>
     </row>
@@ -2182,7 +2561,7 @@
         <v>120</v>
       </c>
       <c r="L17" s="25">
-        <f>(IF(K17-J17&lt;0,0,K17-J17))*G17</f>
+        <f t="shared" si="0"/>
         <v>7.92</v>
       </c>
     </row>
@@ -2221,7 +2600,7 @@
         <v>48</v>
       </c>
       <c r="L18" s="25">
-        <f>(IF(K18-J18&lt;0,0,K18-J18))*G18</f>
+        <f t="shared" si="0"/>
         <v>4.29</v>
       </c>
     </row>
@@ -2260,7 +2639,7 @@
         <v>48</v>
       </c>
       <c r="L19" s="25">
-        <f>(IF(K19-J19&lt;0,0,K19-J19))*G19</f>
+        <f t="shared" si="0"/>
         <v>0.27200000000000002</v>
       </c>
     </row>
@@ -2299,7 +2678,7 @@
         <v>12</v>
       </c>
       <c r="L20" s="25">
-        <f>(IF(K20-J20&lt;0,0,K20-J20))*G20</f>
+        <f t="shared" si="0"/>
         <v>300</v>
       </c>
     </row>
@@ -2338,7 +2717,7 @@
         <v>12</v>
       </c>
       <c r="L21" s="25">
-        <f>(IF(K21-J21&lt;0,0,K21-J21))*G21</f>
+        <f t="shared" si="0"/>
         <v>6.2160000000000002</v>
       </c>
     </row>
@@ -2377,7 +2756,7 @@
         <v>72</v>
       </c>
       <c r="L22" s="25">
-        <f>(IF(K22-J22&lt;0,0,K22-J22))*G22</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2416,7 +2795,7 @@
         <v>72</v>
       </c>
       <c r="L23" s="25">
-        <f>(IF(K23-J23&lt;0,0,K23-J23))*G23</f>
+        <f t="shared" si="0"/>
         <v>36.527999999999999</v>
       </c>
     </row>
@@ -2455,7 +2834,7 @@
         <v>12</v>
       </c>
       <c r="L24" s="25">
-        <f>(IF(K24-J24&lt;0,0,K24-J24))*G24</f>
+        <f t="shared" si="0"/>
         <v>3.9569999999999999</v>
       </c>
     </row>
@@ -2494,7 +2873,7 @@
         <v>360</v>
       </c>
       <c r="L25" s="25">
-        <f>(IF(K25-J25&lt;0,0,K25-J25))*G25</f>
+        <f t="shared" si="0"/>
         <v>31.463999999999999</v>
       </c>
     </row>
@@ -2533,7 +2912,7 @@
         <v>72</v>
       </c>
       <c r="L26" s="25">
-        <f>(IF(K26-J26&lt;0,0,K26-J26))*G26</f>
+        <f t="shared" si="0"/>
         <v>2.044</v>
       </c>
     </row>
@@ -2572,43 +2951,36 @@
         <v>12</v>
       </c>
       <c r="L27" s="25">
-        <f>(IF(K27-J27&lt;0,0,K27-J27))*G27</f>
+        <f t="shared" si="0"/>
         <v>1.5960000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="29"/>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
       <c r="I28" s="13">
         <f>SUM(I2:I27)</f>
         <v>81.931542499999978</v>
       </c>
-      <c r="J28" s="33" t="s">
+      <c r="J28" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="K28" s="33"/>
+      <c r="K28" s="37"/>
       <c r="L28" s="23">
         <f>SUM(L2:L27)</f>
         <v>483.56200000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G31" s="50"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="48"/>
-    </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G32" s="50"/>
-      <c r="H32" s="50"/>
-      <c r="I32" s="49"/>
+      <c r="I32" s="30"/>
     </row>
     <row r="59" ht="31" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="60" ht="32" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2622,7 +2994,7 @@
     <mergeCell ref="C2:C13"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:L27">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>MOD(ROW(),2)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2647,7 +3019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B2A752E-49A0-D348-9E27-6206B0A59C47}">
   <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4331,43 +4703,43 @@
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="B41" s="29"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="29"/>
-      <c r="H41" s="29"/>
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
       <c r="I41" s="23">
         <f>SUM(I2:I40)</f>
         <v>38.513933333333327</v>
       </c>
-      <c r="J41" s="39" t="s">
+      <c r="J41" s="43" t="s">
         <v>209</v>
       </c>
-      <c r="K41" s="39"/>
+      <c r="K41" s="43"/>
       <c r="L41" s="23">
         <f>SUM(L2:L40)</f>
         <v>224.22380000000001</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G44" s="29" t="s">
+      <c r="G44" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="H44" s="29"/>
+      <c r="H44" s="33"/>
       <c r="I44" s="24">
         <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G45" s="29" t="s">
+      <c r="G45" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="29"/>
+      <c r="H45" s="33"/>
       <c r="I45" s="23">
         <f>I41*I44</f>
         <v>462.16719999999992</v>
@@ -4381,7 +4753,7 @@
     <mergeCell ref="J41:K41"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:L40">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>MOD(ROW(),2)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4423,7 +4795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0EFB1B7-3B23-654A-84A7-B98EF9661A5C}">
   <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4483,13 +4855,13 @@
       <c r="B2" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="44" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="41">
+      <c r="E2" s="44">
         <v>29.98</v>
       </c>
       <c r="F2" s="1">
@@ -4503,18 +4875,18 @@
         <v>1</v>
       </c>
       <c r="I2" s="5">
-        <f>H2*G2</f>
+        <f t="shared" ref="I2:I24" si="0">H2*G2</f>
         <v>2.7656550000000002</v>
       </c>
       <c r="J2" s="1">
         <v>0</v>
       </c>
       <c r="K2" s="1">
-        <f>H2*4</f>
+        <f t="shared" ref="K2:K24" si="1">H2*4</f>
         <v>4</v>
       </c>
       <c r="L2" s="5">
-        <f>(IF(K2-J2&lt;0,0,K2-J2))*G2</f>
+        <f t="shared" ref="L2:L24" si="2">(IF(K2-J2&lt;0,0,K2-J2))*G2</f>
         <v>11.062620000000001</v>
       </c>
     </row>
@@ -4525,32 +4897,32 @@
       <c r="B3" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
       <c r="F3" s="1">
         <v>0.17349999999999999</v>
       </c>
       <c r="G3" s="5">
-        <f>F3*E$2/2</f>
+        <f t="shared" ref="G3:G9" si="3">F3*E$2/2</f>
         <v>2.600765</v>
       </c>
       <c r="H3" s="1">
         <v>1</v>
       </c>
       <c r="I3" s="5">
-        <f>H3*G3</f>
+        <f t="shared" si="0"/>
         <v>2.600765</v>
       </c>
       <c r="J3" s="1">
         <v>0</v>
       </c>
       <c r="K3" s="1">
-        <f>H3*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L3" s="5">
-        <f>(IF(K3-J3&lt;0,0,K3-J3))*G3</f>
+        <f t="shared" si="2"/>
         <v>10.40306</v>
       </c>
     </row>
@@ -4561,32 +4933,32 @@
       <c r="B4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="1">
         <v>1.9900000000000001E-2</v>
       </c>
       <c r="G4" s="5">
-        <f>F4*E$2/2</f>
+        <f t="shared" si="3"/>
         <v>0.29830100000000004</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
       </c>
       <c r="I4" s="5">
-        <f>H4*G4</f>
+        <f t="shared" si="0"/>
         <v>0.29830100000000004</v>
       </c>
       <c r="J4" s="1">
         <v>0</v>
       </c>
       <c r="K4" s="1">
-        <f>H4*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L4" s="5">
-        <f>(IF(K4-J4&lt;0,0,K4-J4))*G4</f>
+        <f t="shared" si="2"/>
         <v>1.1932040000000002</v>
       </c>
     </row>
@@ -4597,32 +4969,32 @@
       <c r="B5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
       <c r="F5" s="1">
         <v>6.54E-2</v>
       </c>
       <c r="G5" s="5">
-        <f>F5*E$2/2</f>
+        <f t="shared" si="3"/>
         <v>0.98034600000000005</v>
       </c>
       <c r="H5" s="1">
         <v>1</v>
       </c>
       <c r="I5" s="5">
-        <f>H5*G5</f>
+        <f t="shared" si="0"/>
         <v>0.98034600000000005</v>
       </c>
       <c r="J5" s="1">
         <v>0</v>
       </c>
       <c r="K5" s="1">
-        <f>H5*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L5" s="5">
-        <f>(IF(K5-J5&lt;0,0,K5-J5))*G5</f>
+        <f t="shared" si="2"/>
         <v>3.9213840000000002</v>
       </c>
     </row>
@@ -4633,32 +5005,32 @@
       <c r="B6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
       <c r="F6" s="1">
         <v>0.18579999999999999</v>
       </c>
       <c r="G6" s="5">
-        <f>F6*E$2/2</f>
+        <f t="shared" si="3"/>
         <v>2.785142</v>
       </c>
       <c r="H6" s="1">
         <v>1</v>
       </c>
       <c r="I6" s="5">
-        <f>H6*G6</f>
+        <f t="shared" si="0"/>
         <v>2.785142</v>
       </c>
       <c r="J6" s="1">
         <v>0</v>
       </c>
       <c r="K6" s="1">
-        <f>H6*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L6" s="5">
-        <f>(IF(K6-J6&lt;0,0,K6-J6))*G6</f>
+        <f t="shared" si="2"/>
         <v>11.140568</v>
       </c>
     </row>
@@ -4669,32 +5041,32 @@
       <c r="B7" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="37"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
       <c r="F7" s="1">
         <v>5.9299999999999999E-2</v>
       </c>
       <c r="G7" s="5">
-        <f>F7*E$2/2</f>
+        <f t="shared" si="3"/>
         <v>0.888907</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" s="5">
-        <f>H7*G7</f>
+        <f t="shared" si="0"/>
         <v>0.888907</v>
       </c>
       <c r="J7" s="1">
         <v>0</v>
       </c>
       <c r="K7" s="1">
-        <f>H7*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L7" s="5">
-        <f>(IF(K7-J7&lt;0,0,K7-J7))*G7</f>
+        <f t="shared" si="2"/>
         <v>3.555628</v>
       </c>
     </row>
@@ -4705,32 +5077,32 @@
       <c r="B8" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
       <c r="F8" s="1">
         <v>0.122</v>
       </c>
       <c r="G8" s="5">
-        <f>F8*E$2/2</f>
+        <f t="shared" si="3"/>
         <v>1.8287800000000001</v>
       </c>
       <c r="H8" s="1">
         <v>1</v>
       </c>
       <c r="I8" s="5">
-        <f>H8*G8</f>
+        <f t="shared" si="0"/>
         <v>1.8287800000000001</v>
       </c>
       <c r="J8" s="1">
         <v>0</v>
       </c>
       <c r="K8" s="1">
-        <f>H8*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L8" s="5">
-        <f>(IF(K8-J8&lt;0,0,K8-J8))*G8</f>
+        <f t="shared" si="2"/>
         <v>7.3151200000000003</v>
       </c>
     </row>
@@ -4741,32 +5113,32 @@
       <c r="B9" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="38"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
       <c r="F9" s="1">
         <v>4.3700000000000003E-2</v>
       </c>
       <c r="G9" s="5">
-        <f>F9*E$2/2</f>
+        <f t="shared" si="3"/>
         <v>0.65506300000000006</v>
       </c>
       <c r="H9" s="1">
         <v>2</v>
       </c>
       <c r="I9" s="5">
-        <f>H9*G9</f>
+        <f t="shared" si="0"/>
         <v>1.3101260000000001</v>
       </c>
       <c r="J9" s="1">
         <v>0</v>
       </c>
       <c r="K9" s="1">
-        <f>H9*4</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="L9" s="5">
-        <f>(IF(K9-J9&lt;0,0,K9-J9))*G9</f>
+        <f t="shared" si="2"/>
         <v>5.2405040000000005</v>
       </c>
     </row>
@@ -4796,18 +5168,18 @@
         <v>1</v>
       </c>
       <c r="I10" s="5">
-        <f>H10*G10</f>
+        <f t="shared" si="0"/>
         <v>1.3939999999999999</v>
       </c>
       <c r="J10" s="1">
         <v>0</v>
       </c>
       <c r="K10" s="1">
-        <f>H10*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L10" s="5">
-        <f>(IF(K10-J10&lt;0,0,K10-J10))*G10</f>
+        <f t="shared" si="2"/>
         <v>5.5759999999999996</v>
       </c>
     </row>
@@ -4837,18 +5209,18 @@
         <v>3</v>
       </c>
       <c r="I11" s="5">
-        <f>H11*G11</f>
+        <f t="shared" si="0"/>
         <v>8.4269999999999996</v>
       </c>
       <c r="J11" s="1">
         <v>0</v>
       </c>
       <c r="K11" s="1">
-        <f>H11*4</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="L11" s="5">
-        <f>(IF(K11-J11&lt;0,0,K11-J11))*G11</f>
+        <f t="shared" si="2"/>
         <v>33.707999999999998</v>
       </c>
     </row>
@@ -4878,18 +5250,18 @@
         <v>12</v>
       </c>
       <c r="I12" s="5">
-        <f>H12*G12</f>
+        <f t="shared" si="0"/>
         <v>1.1040000000000001</v>
       </c>
       <c r="J12" s="1">
         <v>0</v>
       </c>
       <c r="K12" s="1">
-        <f>H12*4</f>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="L12" s="5">
-        <f>(IF(K12-J12&lt;0,0,K12-J12))*G12</f>
+        <f t="shared" si="2"/>
         <v>4.4160000000000004</v>
       </c>
     </row>
@@ -4919,18 +5291,18 @@
         <v>2</v>
       </c>
       <c r="I13" s="5">
-        <f>H13*G13</f>
+        <f t="shared" si="0"/>
         <v>0.99199999999999999</v>
       </c>
       <c r="J13" s="1">
         <v>9</v>
       </c>
       <c r="K13" s="1">
-        <f>H13*4</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="L13" s="5">
-        <f>(IF(K13-J13&lt;0,0,K13-J13))*G13</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4960,18 +5332,18 @@
         <v>1</v>
       </c>
       <c r="I14" s="5">
-        <f>H14*G14</f>
+        <f t="shared" si="0"/>
         <v>3.4000000000000002E-2</v>
       </c>
       <c r="J14" s="1">
         <v>0</v>
       </c>
       <c r="K14" s="1">
-        <f>H14*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L14" s="5">
-        <f>(IF(K14-J14&lt;0,0,K14-J14))*G14</f>
+        <f t="shared" si="2"/>
         <v>0.13600000000000001</v>
       </c>
     </row>
@@ -5001,18 +5373,18 @@
         <v>7</v>
       </c>
       <c r="I15" s="5">
-        <f>H15*G15</f>
+        <f t="shared" si="0"/>
         <v>4.8929999999999998</v>
       </c>
       <c r="J15" s="1">
         <v>0</v>
       </c>
       <c r="K15" s="1">
-        <f>H15*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="L15" s="5">
-        <f>(IF(K15-J15&lt;0,0,K15-J15))*G15</f>
+        <f t="shared" si="2"/>
         <v>19.571999999999999</v>
       </c>
     </row>
@@ -5042,18 +5414,18 @@
         <v>7</v>
       </c>
       <c r="I16" s="5">
-        <f>H16*G16</f>
+        <f t="shared" si="0"/>
         <v>1.022</v>
       </c>
       <c r="J16" s="1">
         <v>19</v>
       </c>
       <c r="K16" s="1">
-        <f>H16*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="L16" s="5">
-        <f>(IF(K16-J16&lt;0,0,K16-J16))*G16</f>
+        <f t="shared" si="2"/>
         <v>1.3139999999999998</v>
       </c>
     </row>
@@ -5083,18 +5455,18 @@
         <v>24</v>
       </c>
       <c r="I17" s="5">
-        <f>H17*G17</f>
+        <f t="shared" si="0"/>
         <v>1.6080000000000001</v>
       </c>
       <c r="J17" s="1">
         <v>0</v>
       </c>
       <c r="K17" s="1">
-        <f>H17*4</f>
+        <f t="shared" si="1"/>
         <v>96</v>
       </c>
       <c r="L17" s="5">
-        <f>(IF(K17-J17&lt;0,0,K17-J17))*G17</f>
+        <f t="shared" si="2"/>
         <v>6.4320000000000004</v>
       </c>
     </row>
@@ -5124,18 +5496,18 @@
         <v>7</v>
       </c>
       <c r="I18" s="5">
-        <f>H18*G18</f>
+        <f t="shared" si="0"/>
         <v>2.2400000000000002</v>
       </c>
       <c r="J18" s="1">
         <v>0</v>
       </c>
       <c r="K18" s="1">
-        <f>H18*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="L18" s="5">
-        <f>(IF(K18-J18&lt;0,0,K18-J18))*G18</f>
+        <f t="shared" si="2"/>
         <v>8.9600000000000009</v>
       </c>
     </row>
@@ -5165,18 +5537,18 @@
         <v>5</v>
       </c>
       <c r="I19" s="5">
-        <f>H19*G19</f>
+        <f t="shared" si="0"/>
         <v>4.1449999999999996</v>
       </c>
       <c r="J19" s="1">
         <v>10</v>
       </c>
       <c r="K19" s="1">
-        <f>H19*4</f>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="L19" s="5">
-        <f>(IF(K19-J19&lt;0,0,K19-J19))*G19</f>
+        <f t="shared" si="2"/>
         <v>8.2899999999999991</v>
       </c>
     </row>
@@ -5206,18 +5578,18 @@
         <v>1</v>
       </c>
       <c r="I20" s="5">
-        <f>H20*G20</f>
+        <f t="shared" si="0"/>
         <v>0.53800000000000003</v>
       </c>
       <c r="J20" s="1">
         <v>0</v>
       </c>
       <c r="K20" s="1">
-        <f>H20*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L20" s="5">
-        <f>(IF(K20-J20&lt;0,0,K20-J20))*G20</f>
+        <f t="shared" si="2"/>
         <v>2.1520000000000001</v>
       </c>
     </row>
@@ -5247,18 +5619,18 @@
         <v>3</v>
       </c>
       <c r="I21" s="5">
-        <f>H21*G21</f>
+        <f t="shared" si="0"/>
         <v>0.153</v>
       </c>
       <c r="J21" s="1">
         <v>40</v>
       </c>
       <c r="K21" s="1">
-        <f>H21*4</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="L21" s="5">
-        <f>(IF(K21-J21&lt;0,0,K21-J21))*G21</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5288,18 +5660,18 @@
         <v>1</v>
       </c>
       <c r="I22" s="5">
-        <f>H22*G22</f>
+        <f t="shared" si="0"/>
         <v>0.221</v>
       </c>
       <c r="J22" s="1">
         <v>0</v>
       </c>
       <c r="K22" s="1">
-        <f>H22*4</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="L22" s="5">
-        <f>(IF(K22-J22&lt;0,0,K22-J22))*G22</f>
+        <f t="shared" si="2"/>
         <v>0.88400000000000001</v>
       </c>
     </row>
@@ -5329,18 +5701,18 @@
         <v>3</v>
       </c>
       <c r="I23" s="5">
-        <f>H23*G23</f>
+        <f t="shared" si="0"/>
         <v>0.84599999999999986</v>
       </c>
       <c r="J23" s="1">
         <v>15</v>
       </c>
       <c r="K23" s="1">
-        <f>H23*4</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="L23" s="5">
-        <f>(IF(K23-J23&lt;0,0,K23-J23))*G23</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5370,49 +5742,49 @@
         <v>18</v>
       </c>
       <c r="I24" s="5">
-        <f>H24*G24</f>
+        <f t="shared" si="0"/>
         <v>1.3499999999999999</v>
       </c>
       <c r="J24" s="1">
         <v>10</v>
       </c>
       <c r="K24" s="1">
-        <f>H24*4</f>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
       <c r="L24" s="5">
-        <f>(IF(K24-J24&lt;0,0,K24-J24))*G24</f>
+        <f t="shared" si="2"/>
         <v>4.6499999999999995</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="47">
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47"/>
+      <c r="G25" s="47"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="29">
         <f>SUM(I2:I24)</f>
         <v>42.425021999999984</v>
       </c>
-      <c r="J25" s="42" t="s">
+      <c r="J25" s="49" t="s">
         <v>209</v>
       </c>
-      <c r="K25" s="43"/>
-      <c r="L25" s="47">
+      <c r="K25" s="50"/>
+      <c r="L25" s="29">
         <f>SUM(L2:L24)</f>
         <v>149.92208799999995</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="J28" s="51"/>
-      <c r="K28" s="51"/>
-      <c r="L28" s="52"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5422,7 +5794,7 @@
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="J25:K25"/>
   </mergeCells>
-  <conditionalFormatting sqref="A2:L2 A3:B9 F3:J9 A10:J24 K3:L24">
+  <conditionalFormatting sqref="A2:L2 A3:B9 F3:J9 K3:L24 A10:J24">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>MOD(ROW(),2)</formula>
     </cfRule>

</xml_diff>